<commit_message>
more testing data added for non-uk locations
</commit_message>
<xml_diff>
--- a/data/schemes_input.xlsx
+++ b/data/schemes_input.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://staticus-my.sharepoint.com/personal/orlin_kolev_staticus_com/Documents/Desktop/Jobs/2026 03 WinLoad automation/current version/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://staticus-my.sharepoint.com/personal/orlin_kolev_staticus_com/Documents/Desktop/Jobs/WinLoad automation/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_2B4385C93F55C2CC17B90BED6C790FE2E1A0DFE7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2E822F8C-27EC-48AC-BBA9-F02C82E62479}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="11_2B4385C93F55C2CC17B90BED6C790FE2E1A0DFE7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D930CE1-A2A1-459D-BE1B-37DC41A86672}"/>
   <bookViews>
-    <workbookView xWindow="3072" yWindow="624" windowWidth="26064" windowHeight="16656" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="384" yWindow="384" windowWidth="27036" windowHeight="16656" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Schemes" sheetId="1" r:id="rId1"/>
@@ -464,7 +464,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.3">
@@ -528,9 +528,49 @@
         <v>40</v>
       </c>
       <c r="F2">
+        <v>50.496068747232798</v>
+      </c>
+      <c r="G2">
+        <v>11.2427773401017</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>30</v>
+      </c>
+      <c r="D3">
+        <v>20</v>
+      </c>
+      <c r="E3">
+        <v>40</v>
+      </c>
+      <c r="F3">
+        <v>42.705052028942099</v>
+      </c>
+      <c r="G3">
+        <v>23.306286012708</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="C4">
+        <v>30</v>
+      </c>
+      <c r="D4">
+        <v>20</v>
+      </c>
+      <c r="E4">
+        <v>40</v>
+      </c>
+      <c r="F4">
         <v>53.797857</v>
       </c>
-      <c r="G2">
+      <c r="G4">
         <v>-1.5577669999999999</v>
       </c>
     </row>

</xml_diff>